<commit_message>
jul3 removed combined calc
</commit_message>
<xml_diff>
--- a/testing_electricity_202604_highlighted.xlsx
+++ b/testing_electricity_202604_highlighted.xlsx
@@ -28287,7 +28287,7 @@
       <c r="H148" s="168" t="n">
         <v>335356</v>
       </c>
-      <c r="I148" s="304" t="n">
+      <c r="I148" s="168" t="n">
         <v>620519</v>
       </c>
       <c r="J148" s="168" t="n">
@@ -28342,7 +28342,7 @@
       <c r="AA148" s="168" t="n">
         <v>281582</v>
       </c>
-      <c r="AB148" s="168" t="n">
+      <c r="AB148" s="304" t="n">
         <v>665379</v>
       </c>
       <c r="AD148" s="168" t="n">

</xml_diff>

<commit_message>
jul6 yaml + waste trial
- adapted yaml
- changed checking data range from basing on today to last month that updates in source
- created yaml template and tested on nixon waste reports
- fixed convert tonnes to kg (this took 2 hours)
</commit_message>
<xml_diff>
--- a/testing_electricity_202604_highlighted.xlsx
+++ b/testing_electricity_202604_highlighted.xlsx
@@ -27553,7 +27553,7 @@
       <c r="AH140" s="49" t="n">
         <v>14241.92</v>
       </c>
-      <c r="AI140" s="49" t="n">
+      <c r="AI140" s="304" t="n">
         <v>32039</v>
       </c>
     </row>
@@ -27653,7 +27653,7 @@
       <c r="AH141" s="49" t="n">
         <v>14634.33</v>
       </c>
-      <c r="AI141" s="49" t="n">
+      <c r="AI141" s="304" t="n">
         <v>41319</v>
       </c>
     </row>

</xml_diff>